<commit_message>
error rasgos Bombuscaro, outliers, graphs
</commit_message>
<xml_diff>
--- a/Results_isofys/05. Rasgos_Bombuscaro_Cajanuma.xlsx
+++ b/Results_isofys/05. Rasgos_Bombuscaro_Cajanuma.xlsx
@@ -619,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -630,6 +630,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -845,11 +847,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AF1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="8.7109375" customWidth="1"/>
+    <col min="1" max="2" width="4.42578125" customWidth="1"/>
+    <col min="3" max="5" width="8.7109375" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" customWidth="1"/>
     <col min="8" max="8" width="8.28515625" customWidth="1"/>
@@ -3157,7 +3159,7 @@
       <c r="F26" s="4">
         <v>45617</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="7" t="s">
         <v>71</v>
       </c>
       <c r="I26" s="3" t="s">
@@ -3220,11 +3222,11 @@
       <c r="AB26" s="3">
         <v>20</v>
       </c>
-      <c r="AC26" s="3">
-        <v>34.11</v>
-      </c>
-      <c r="AD26" s="3">
-        <v>18.97</v>
+      <c r="AC26" s="6">
+        <v>30</v>
+      </c>
+      <c r="AD26" s="7">
+        <v>16.690000000000001</v>
       </c>
       <c r="AE26" s="3" t="s">
         <v>72</v>
@@ -3252,7 +3254,7 @@
       <c r="F27" s="4">
         <v>45617</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="7" t="s">
         <v>73</v>
       </c>
       <c r="I27" s="3" t="s">
@@ -3312,11 +3314,11 @@
       <c r="AB27" s="3">
         <v>20</v>
       </c>
-      <c r="AC27" s="3">
-        <v>38.97</v>
-      </c>
-      <c r="AD27" s="3">
-        <v>18.77</v>
+      <c r="AC27" s="7">
+        <v>34.11</v>
+      </c>
+      <c r="AD27" s="7">
+        <v>18.97</v>
       </c>
       <c r="AE27" s="3" t="s">
         <v>74</v>
@@ -3344,7 +3346,7 @@
       <c r="F28" s="4">
         <v>45617</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="7" t="s">
         <v>75</v>
       </c>
       <c r="I28" s="3" t="s">
@@ -3407,11 +3409,11 @@
       <c r="AB28" s="3">
         <v>20</v>
       </c>
-      <c r="AC28" s="3">
-        <v>30.07</v>
-      </c>
-      <c r="AD28" s="3">
-        <v>15.23</v>
+      <c r="AC28" s="7">
+        <v>38.97</v>
+      </c>
+      <c r="AD28" s="7">
+        <v>18.77</v>
       </c>
       <c r="AF28" s="3">
         <v>1332.5820000000001</v>
@@ -3436,7 +3438,7 @@
       <c r="F29" s="4">
         <v>45617</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H29" s="3" t="s">
@@ -3499,11 +3501,11 @@
       <c r="AB29" s="3">
         <v>20</v>
       </c>
-      <c r="AC29" s="3">
-        <v>14.55</v>
-      </c>
-      <c r="AD29" s="3">
-        <v>5.69</v>
+      <c r="AC29" s="7">
+        <v>30.07</v>
+      </c>
+      <c r="AD29" s="7">
+        <v>15.23</v>
       </c>
       <c r="AF29" s="3">
         <v>1248.499</v>
@@ -3528,7 +3530,7 @@
       <c r="F30" s="4">
         <v>45617</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="7" t="s">
         <v>78</v>
       </c>
       <c r="H30" s="3">
@@ -3591,11 +3593,11 @@
       <c r="AB30" s="3">
         <v>20</v>
       </c>
-      <c r="AC30" s="3">
-        <v>30</v>
-      </c>
-      <c r="AD30" s="3">
-        <v>16.690000000000001</v>
+      <c r="AC30" s="7">
+        <v>14.55</v>
+      </c>
+      <c r="AD30" s="7">
+        <v>5.69</v>
       </c>
       <c r="AF30" s="3">
         <v>579.08100000000002</v>
@@ -4405,7 +4407,7 @@
         <v>20</v>
       </c>
       <c r="AC39" s="3">
-        <v>25.15</v>
+        <v>35.15</v>
       </c>
       <c r="AD39" s="3">
         <v>18.2</v>
@@ -4494,7 +4496,7 @@
         <v>20</v>
       </c>
       <c r="AC40" s="3">
-        <v>25.52</v>
+        <v>35.520000000000003</v>
       </c>
       <c r="AD40" s="3">
         <v>17.36</v>
@@ -5239,7 +5241,7 @@
         <v>176.61370529999999</v>
       </c>
     </row>
-    <row r="49" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -5331,7 +5333,7 @@
         <v>31.193000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -5423,7 +5425,7 @@
         <v>34.548281500000002</v>
       </c>
     </row>
-    <row r="51" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -5515,7 +5517,7 @@
         <v>41.29</v>
       </c>
     </row>
-    <row r="52" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -5607,7 +5609,7 @@
         <v>37.481708599999997</v>
       </c>
     </row>
-    <row r="53" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -5699,7 +5701,7 @@
         <v>25.962922299999999</v>
       </c>
     </row>
-    <row r="54" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -6818,7 +6820,7 @@
         <v>363.37691890000002</v>
       </c>
     </row>
-    <row r="66" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -6910,7 +6912,7 @@
         <v>30.444854299999999</v>
       </c>
     </row>
-    <row r="67" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -7002,7 +7004,7 @@
         <v>37.5134951</v>
       </c>
     </row>
-    <row r="68" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -7278,7 +7280,7 @@
         <v>400.27849179999998</v>
       </c>
     </row>
-    <row r="71" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -7370,7 +7372,7 @@
         <v>33.473779800000003</v>
       </c>
     </row>
-    <row r="72" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -7462,7 +7464,7 @@
         <v>57.475637399999997</v>
       </c>
     </row>
-    <row r="73" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -7646,7 +7648,7 @@
         <v>431.89406120000001</v>
       </c>
     </row>
-    <row r="75" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -7830,7 +7832,7 @@
         <v>404.1618411</v>
       </c>
     </row>
-    <row r="77" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -8106,7 +8108,7 @@
         <v>418.39213590000003</v>
       </c>
     </row>
-    <row r="80" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>78</v>
       </c>
@@ -8198,7 +8200,7 @@
         <v>28.873925499999999</v>
       </c>
     </row>
-    <row r="81" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>79</v>
       </c>
@@ -8379,7 +8381,7 @@
         <v>250.358</v>
       </c>
     </row>
-    <row r="83" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>81</v>
       </c>
@@ -8471,7 +8473,7 @@
         <v>35.679000000000002</v>
       </c>
     </row>
-    <row r="84" spans="1:32" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>82</v>
       </c>
@@ -9480,11 +9482,6 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AF84">
-    <filterColumn colId="11">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>